<commit_message>
atualização com filter direto do XLSX e filter --clear-users
</commit_message>
<xml_diff>
--- a/contratos_ativos.xlsx
+++ b/contratos_ativos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tarcisio.maciel\Documents\GM GROUP\Data Engineer\LakeHouse\Assuntos\Data Migration - CORE from ERP\app_migracao_core\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE6F0445-E5F8-48EF-916F-F0F233BB0079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E5BD47-0F34-4EA9-8519-834A47BD50F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{457C6F6E-1596-43CA-A196-F52A8B728ADA}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Clientes_2026_03_13" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Clientes_2026_03_13!$A$1:$Q$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Clientes_2026_03_13!$A$1:$R$204</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -782,7 +782,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -842,6 +842,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -884,7 +898,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -960,6 +974,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1339,6 +1362,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64C195D-2B79-4C6D-852C-4F0C248DE140}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R204"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2172,38 +2196,38 @@
       <c r="G16" s="9">
         <v>6042467000180</v>
       </c>
-      <c r="H16" s="7">
-        <v>1</v>
-      </c>
-      <c r="I16" s="7">
+      <c r="H16" s="29">
+        <v>1</v>
+      </c>
+      <c r="I16" s="29">
         <v>20</v>
       </c>
-      <c r="J16" s="7">
-        <v>0</v>
-      </c>
-      <c r="K16" t="s">
+      <c r="J16" s="29">
+        <v>0</v>
+      </c>
+      <c r="K16" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="L16" s="10">
-        <v>46123</v>
-      </c>
-      <c r="M16" s="6">
-        <v>46094</v>
-      </c>
-      <c r="N16" t="s">
+      <c r="L16" s="31">
+        <v>46123</v>
+      </c>
+      <c r="M16" s="32">
+        <v>46094</v>
+      </c>
+      <c r="N16" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="O16" t="s">
-        <v>22</v>
-      </c>
-      <c r="P16" s="13">
+      <c r="O16" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="P16" s="33">
         <v>46067401835</v>
       </c>
-      <c r="Q16" s="13">
+      <c r="Q16" s="33">
         <v>46067401835</v>
       </c>
       <c r="R16" s="8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
@@ -9583,7 +9607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="14">
         <v>7014</v>
       </c>
@@ -9639,7 +9663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="14">
         <v>5512</v>
       </c>
@@ -9695,7 +9719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="14">
         <v>11044</v>
       </c>
@@ -9747,7 +9771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="14">
         <v>7877</v>
       </c>
@@ -9803,7 +9827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="14">
         <v>3284</v>
       </c>
@@ -9859,7 +9883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="14">
         <v>11825</v>
       </c>
@@ -9915,7 +9939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="14">
         <v>13722</v>
       </c>
@@ -9963,7 +9987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="14">
         <v>11815</v>
       </c>
@@ -10019,7 +10043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="14">
         <v>7286</v>
       </c>
@@ -10075,7 +10099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="14">
         <v>11822</v>
       </c>
@@ -10123,7 +10147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="14">
         <v>13672</v>
       </c>
@@ -10179,7 +10203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="14">
         <v>9343</v>
       </c>
@@ -10235,7 +10259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="14">
         <v>13925</v>
       </c>
@@ -10283,7 +10307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="14">
         <v>8854</v>
       </c>
@@ -10386,10 +10410,10 @@
         <v>39183725881</v>
       </c>
       <c r="R166" s="8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="167" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="14">
         <v>4968</v>
       </c>
@@ -10445,7 +10469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="14">
         <v>13619</v>
       </c>
@@ -10501,7 +10525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="14">
         <v>8355</v>
       </c>
@@ -10557,7 +10581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="14">
         <v>11813</v>
       </c>
@@ -10613,7 +10637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="14">
         <v>6554</v>
       </c>
@@ -10669,7 +10693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="14">
         <v>13646</v>
       </c>
@@ -10725,7 +10749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="14">
         <v>11817</v>
       </c>
@@ -10781,7 +10805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="14">
         <v>13526</v>
       </c>
@@ -10837,7 +10861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="14">
         <v>5961</v>
       </c>
@@ -10893,7 +10917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="14">
         <v>10735</v>
       </c>
@@ -10949,7 +10973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="14">
         <v>13780</v>
       </c>
@@ -11001,7 +11025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="14">
         <v>17</v>
       </c>
@@ -11057,7 +11081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="14">
         <v>7125</v>
       </c>
@@ -11113,7 +11137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="14">
         <v>7714</v>
       </c>
@@ -11169,7 +11193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="14">
         <v>8261</v>
       </c>
@@ -11225,7 +11249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="14">
         <v>13902</v>
       </c>
@@ -11273,7 +11297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="14">
         <v>13764</v>
       </c>
@@ -11325,7 +11349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="14">
         <v>13624</v>
       </c>
@@ -11375,7 +11399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="14">
         <v>13502</v>
       </c>
@@ -11431,7 +11455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="14">
         <v>5341</v>
       </c>
@@ -11487,7 +11511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="14">
         <v>11858</v>
       </c>
@@ -11543,7 +11567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="14">
         <v>7916</v>
       </c>
@@ -11595,7 +11619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="14">
         <v>13788</v>
       </c>
@@ -11647,7 +11671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="14">
         <v>4939</v>
       </c>
@@ -11703,7 +11727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14">
         <v>6793</v>
       </c>
@@ -11759,7 +11783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="14">
         <v>7737</v>
       </c>
@@ -11815,7 +11839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="14">
         <v>11831</v>
       </c>
@@ -11871,7 +11895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="14">
         <v>13708</v>
       </c>
@@ -11923,7 +11947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="14">
         <v>6912</v>
       </c>
@@ -11979,7 +12003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="14">
         <v>12923</v>
       </c>
@@ -12031,7 +12055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="14">
         <v>13882</v>
       </c>
@@ -12079,7 +12103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="14">
         <v>11261</v>
       </c>
@@ -12135,7 +12159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14">
         <v>10709</v>
       </c>
@@ -12191,7 +12215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="14">
         <v>2593</v>
       </c>
@@ -12247,7 +12271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="14">
         <v>4973</v>
       </c>
@@ -12303,7 +12327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="14">
         <v>11221</v>
       </c>
@@ -12359,7 +12383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="14">
         <v>13678</v>
       </c>
@@ -12411,7 +12435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="14">
         <v>11049</v>
       </c>
@@ -12468,6 +12492,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:R204" xr:uid="{C64C195D-2B79-4C6D-852C-4F0C248DE140}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="VERDADEIRO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q204">
     <sortCondition descending="1" ref="F2:F204"/>
   </sortState>

</xml_diff>

<commit_message>
HML funcionando perfeitamente. Próximo passo, ajustar sem o comando CLEAR DATA
</commit_message>
<xml_diff>
--- a/contratos_ativos.xlsx
+++ b/contratos_ativos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tarcisio.maciel\Documents\GM GROUP\Data Engineer\LakeHouse\Assuntos\Data Migration - CORE from ERP\app_migracao_core\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E5BD47-0F34-4EA9-8519-834A47BD50F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1AD18B2-CF1C-422C-8A1A-8BBC2D4B0E88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{457C6F6E-1596-43CA-A196-F52A8B728ADA}"/>
   </bookViews>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="229">
   <si>
     <t>ORÇAMENTO</t>
   </si>
@@ -773,6 +773,9 @@
   </si>
   <si>
     <t>VOLK DO BRASIL</t>
+  </si>
+  <si>
+    <t>NO CHARGE</t>
   </si>
 </sst>
 </file>
@@ -1441,7 +1444,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>13632</v>
       </c>
@@ -1497,7 +1500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>6605</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>13717</v>
       </c>
@@ -1603,7 +1606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>13686</v>
       </c>
@@ -1659,9 +1662,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>1309313093</v>
+        <v>13093</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
@@ -1715,7 +1718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5130</v>
       </c>
@@ -1771,7 +1774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>13838</v>
       </c>
@@ -1821,7 +1824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5670</v>
       </c>
@@ -1877,7 +1880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>13872</v>
       </c>
@@ -1921,7 +1924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>13905</v>
       </c>
@@ -1968,7 +1971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>13856</v>
       </c>
@@ -2018,7 +2021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5191</v>
       </c>
@@ -2074,7 +2077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13207</v>
       </c>
@@ -2124,7 +2127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13177</v>
       </c>
@@ -2174,7 +2177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>13520</v>
       </c>
@@ -2227,10 +2230,10 @@
         <v>46067401835</v>
       </c>
       <c r="R16" s="8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13903</v>
       </c>
@@ -2277,7 +2280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>13751</v>
       </c>
@@ -2327,7 +2330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>13797</v>
       </c>
@@ -2377,7 +2380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>5672</v>
       </c>
@@ -2433,7 +2436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>6991</v>
       </c>
@@ -2489,7 +2492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>13851</v>
       </c>
@@ -2539,7 +2542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>11820</v>
       </c>
@@ -2595,7 +2598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>7804</v>
       </c>
@@ -2651,7 +2654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>9138</v>
       </c>
@@ -2754,10 +2757,10 @@
         <v>73368172549</v>
       </c>
       <c r="R26" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>13512</v>
       </c>
@@ -2807,7 +2810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>8994</v>
       </c>
@@ -2863,7 +2866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>11830</v>
       </c>
@@ -2919,7 +2922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>13276</v>
       </c>
@@ -2975,7 +2978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>8257</v>
       </c>
@@ -3031,7 +3034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>13179</v>
       </c>
@@ -3087,7 +3090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>11848</v>
       </c>
@@ -3131,7 +3134,7 @@
         <v>29</v>
       </c>
       <c r="O33" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P33" s="13">
         <v>46067401835</v>
@@ -3143,7 +3146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>8599</v>
       </c>
@@ -3199,7 +3202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>6699</v>
       </c>
@@ -3255,7 +3258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>13747</v>
       </c>
@@ -3302,7 +3305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>13878</v>
       </c>
@@ -3349,7 +3352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>13914</v>
       </c>
@@ -3396,7 +3399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>10412</v>
       </c>
@@ -3452,7 +3455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>13076</v>
       </c>
@@ -3508,7 +3511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>13618</v>
       </c>
@@ -3564,7 +3567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>13447</v>
       </c>
@@ -3620,7 +3623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:18" s="22" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" s="22" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="22">
         <v>11844</v>
       </c>
@@ -3664,7 +3667,7 @@
         <v>21</v>
       </c>
       <c r="O43" s="22" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P43" s="28">
         <v>39183725881</v>
@@ -3676,7 +3679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>224</v>
       </c>
@@ -3720,7 +3723,7 @@
         <v>21</v>
       </c>
       <c r="O44" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P44" s="13">
         <v>15149756881</v>
@@ -3776,7 +3779,7 @@
         <v>21</v>
       </c>
       <c r="O45" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P45" s="13">
         <v>35538393844</v>
@@ -3785,10 +3788,10 @@
         <v>35538393844</v>
       </c>
       <c r="R45" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>6816</v>
       </c>
@@ -3832,7 +3835,7 @@
         <v>21</v>
       </c>
       <c r="O46" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P46" s="13">
         <v>35538393844</v>
@@ -3844,7 +3847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>5696</v>
       </c>
@@ -3888,7 +3891,7 @@
         <v>21</v>
       </c>
       <c r="O47" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P47" s="13">
         <v>73368172549</v>
@@ -3900,7 +3903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>8892</v>
       </c>
@@ -3944,7 +3947,7 @@
         <v>21</v>
       </c>
       <c r="O48" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P48" s="13">
         <v>33615887824</v>
@@ -3956,7 +3959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>7969</v>
       </c>
@@ -4000,7 +4003,7 @@
         <v>29</v>
       </c>
       <c r="O49" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P49" s="13">
         <v>15149756881</v>
@@ -4012,7 +4015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>6772</v>
       </c>
@@ -4056,7 +4059,7 @@
         <v>21</v>
       </c>
       <c r="O50" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P50" s="13">
         <v>46067401835</v>
@@ -4112,7 +4115,7 @@
         <v>29</v>
       </c>
       <c r="O51" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P51" s="13">
         <v>39183725881</v>
@@ -4121,10 +4124,10 @@
         <v>39183725881</v>
       </c>
       <c r="R51" s="8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>11243</v>
       </c>
@@ -4168,7 +4171,7 @@
         <v>21</v>
       </c>
       <c r="O52" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P52" s="13">
         <v>33615887824</v>
@@ -4180,7 +4183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>8609</v>
       </c>
@@ -4224,7 +4227,7 @@
         <v>21</v>
       </c>
       <c r="O53" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P53" s="13">
         <v>35884552807</v>
@@ -4236,7 +4239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>11174</v>
       </c>
@@ -4280,7 +4283,7 @@
         <v>21</v>
       </c>
       <c r="O54" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P54" s="13">
         <v>15149756881</v>
@@ -4292,7 +4295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>13642</v>
       </c>
@@ -4330,7 +4333,7 @@
         <v>21</v>
       </c>
       <c r="O55" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P55" s="13">
         <v>35538393844</v>
@@ -4342,7 +4345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>13288</v>
       </c>
@@ -4386,7 +4389,7 @@
         <v>21</v>
       </c>
       <c r="O56" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P56" s="13">
         <v>39183725881</v>
@@ -4398,7 +4401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>11812</v>
       </c>
@@ -4442,7 +4445,7 @@
         <v>21</v>
       </c>
       <c r="O57" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P57" s="13">
         <v>33615887824</v>
@@ -4454,7 +4457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>13931</v>
       </c>
@@ -4492,7 +4495,7 @@
         <v>21</v>
       </c>
       <c r="O58" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P58" s="13" t="s">
         <v>38</v>
@@ -4504,7 +4507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>7758</v>
       </c>
@@ -4548,7 +4551,7 @@
         <v>21</v>
       </c>
       <c r="O59" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P59" s="13">
         <v>35884552807</v>
@@ -4560,7 +4563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>6824</v>
       </c>
@@ -4604,7 +4607,7 @@
         <v>21</v>
       </c>
       <c r="O60" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P60" s="13">
         <v>46067401835</v>
@@ -4616,7 +4619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>10999</v>
       </c>
@@ -4660,7 +4663,7 @@
         <v>21</v>
       </c>
       <c r="O61" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P61" s="13">
         <v>33615887824</v>
@@ -4672,7 +4675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>1418</v>
       </c>
@@ -4716,7 +4719,7 @@
         <v>21</v>
       </c>
       <c r="O62" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P62" s="13">
         <v>39183725881</v>
@@ -4728,7 +4731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>13236</v>
       </c>
@@ -4772,7 +4775,7 @@
         <v>21</v>
       </c>
       <c r="O63" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P63" s="13">
         <v>46067401835</v>
@@ -4784,7 +4787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:18" s="22" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" s="22" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="22">
         <v>13265</v>
       </c>
@@ -4828,7 +4831,7 @@
         <v>45</v>
       </c>
       <c r="O64" s="22" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P64" s="28">
         <v>73368172549</v>
@@ -4840,7 +4843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>5349</v>
       </c>
@@ -4878,7 +4881,7 @@
         <v>21</v>
       </c>
       <c r="O65" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P65" s="13">
         <v>15149756881</v>
@@ -4890,7 +4893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>6697</v>
       </c>
@@ -4934,7 +4937,7 @@
         <v>21</v>
       </c>
       <c r="O66" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P66" s="13">
         <v>73368172549</v>
@@ -4946,7 +4949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>13803</v>
       </c>
@@ -4984,7 +4987,7 @@
         <v>45</v>
       </c>
       <c r="O67" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P67" s="13">
         <v>35884552807</v>
@@ -4996,7 +4999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>13711</v>
       </c>
@@ -5034,7 +5037,7 @@
         <v>21</v>
       </c>
       <c r="O68" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P68" s="13">
         <v>39183725881</v>
@@ -5046,7 +5049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>8065</v>
       </c>
@@ -5090,7 +5093,7 @@
         <v>21</v>
       </c>
       <c r="O69" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P69" s="13" t="s">
         <v>38</v>
@@ -5102,7 +5105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>13707</v>
       </c>
@@ -5146,7 +5149,7 @@
         <v>21</v>
       </c>
       <c r="O70" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P70" s="13">
         <v>33615887824</v>
@@ -5158,7 +5161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>5674</v>
       </c>
@@ -5202,7 +5205,7 @@
         <v>21</v>
       </c>
       <c r="O71" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P71" s="13">
         <v>33615887824</v>
@@ -5214,7 +5217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>13575</v>
       </c>
@@ -5252,7 +5255,7 @@
         <v>29</v>
       </c>
       <c r="O72" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P72" s="13">
         <v>35884552807</v>
@@ -5264,7 +5267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>11819</v>
       </c>
@@ -5308,7 +5311,7 @@
         <v>21</v>
       </c>
       <c r="O73" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P73" s="13">
         <v>15149756881</v>
@@ -5320,7 +5323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>12925</v>
       </c>
@@ -5364,7 +5367,7 @@
         <v>21</v>
       </c>
       <c r="O74" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P74" s="13">
         <v>15149756881</v>
@@ -5376,7 +5379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>6583</v>
       </c>
@@ -5420,7 +5423,7 @@
         <v>21</v>
       </c>
       <c r="O75" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P75" s="13">
         <v>39183725881</v>
@@ -5432,7 +5435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>6579</v>
       </c>
@@ -5476,7 +5479,7 @@
         <v>21</v>
       </c>
       <c r="O76" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P76" s="13">
         <v>73368172549</v>
@@ -5488,7 +5491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>13174</v>
       </c>
@@ -5532,7 +5535,7 @@
         <v>29</v>
       </c>
       <c r="O77" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P77" s="13">
         <v>73368172549</v>
@@ -5544,7 +5547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2105</v>
       </c>
@@ -5588,7 +5591,7 @@
         <v>29</v>
       </c>
       <c r="O78" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P78" s="13">
         <v>73368172549</v>
@@ -5600,7 +5603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>13474</v>
       </c>
@@ -5638,7 +5641,7 @@
         <v>45</v>
       </c>
       <c r="O79" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P79" s="13">
         <v>39183725881</v>
@@ -5650,7 +5653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>13727</v>
       </c>
@@ -5688,7 +5691,7 @@
         <v>21</v>
       </c>
       <c r="O80" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P80" s="13">
         <v>39183725881</v>
@@ -5700,7 +5703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>13504</v>
       </c>
@@ -5744,7 +5747,7 @@
         <v>21</v>
       </c>
       <c r="O81" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P81" s="13">
         <v>73368172549</v>
@@ -5756,7 +5759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>13551</v>
       </c>
@@ -5800,7 +5803,7 @@
         <v>21</v>
       </c>
       <c r="O82" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P82" s="13">
         <v>35884552807</v>
@@ -5812,7 +5815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>11826</v>
       </c>
@@ -5856,7 +5859,7 @@
         <v>21</v>
       </c>
       <c r="O83" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P83" s="13">
         <v>15149756881</v>
@@ -5868,7 +5871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>13486</v>
       </c>
@@ -5906,7 +5909,7 @@
         <v>21</v>
       </c>
       <c r="O84" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P84" s="13">
         <v>46067401835</v>
@@ -5918,7 +5921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>5539</v>
       </c>
@@ -5962,7 +5965,7 @@
         <v>21</v>
       </c>
       <c r="O85" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P85" s="13">
         <v>46067401835</v>
@@ -5974,7 +5977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>9244</v>
       </c>
@@ -6018,7 +6021,7 @@
         <v>21</v>
       </c>
       <c r="O86" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P86" s="13">
         <v>73368172549</v>
@@ -6030,7 +6033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>13830</v>
       </c>
@@ -6068,7 +6071,7 @@
         <v>21</v>
       </c>
       <c r="O87" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P87" s="13">
         <v>73368172549</v>
@@ -6080,7 +6083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>13688</v>
       </c>
@@ -6124,7 +6127,7 @@
         <v>21</v>
       </c>
       <c r="O88" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P88" s="13">
         <v>15149756881</v>
@@ -6136,7 +6139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>13580</v>
       </c>
@@ -6180,7 +6183,7 @@
         <v>21</v>
       </c>
       <c r="O89" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P89" s="13">
         <v>39183725881</v>
@@ -6192,7 +6195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>6053</v>
       </c>
@@ -6236,7 +6239,7 @@
         <v>21</v>
       </c>
       <c r="O90" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P90" s="13">
         <v>33615887824</v>
@@ -6248,7 +6251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>13874</v>
       </c>
@@ -6286,7 +6289,7 @@
         <v>21</v>
       </c>
       <c r="O91" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P91" s="13">
         <v>46067401835</v>
@@ -6298,7 +6301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>13880</v>
       </c>
@@ -6336,7 +6339,7 @@
         <v>21</v>
       </c>
       <c r="O92" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P92" s="13" t="s">
         <v>38</v>
@@ -6345,7 +6348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>10966</v>
       </c>
@@ -6389,7 +6392,7 @@
         <v>29</v>
       </c>
       <c r="O93" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P93" s="13">
         <v>35884552807</v>
@@ -6401,7 +6404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>7976</v>
       </c>
@@ -6445,7 +6448,7 @@
         <v>29</v>
       </c>
       <c r="O94" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P94" s="13">
         <v>35884552807</v>
@@ -6457,7 +6460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>9196</v>
       </c>
@@ -6501,7 +6504,7 @@
         <v>21</v>
       </c>
       <c r="O95" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P95" s="13">
         <v>39183725881</v>
@@ -6513,7 +6516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>8782</v>
       </c>
@@ -6557,7 +6560,7 @@
         <v>21</v>
       </c>
       <c r="O96" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P96" s="13">
         <v>33615887824</v>
@@ -6569,7 +6572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>8119</v>
       </c>
@@ -6613,7 +6616,7 @@
         <v>21</v>
       </c>
       <c r="O97" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P97" s="13">
         <v>73368172549</v>
@@ -6625,7 +6628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>5376</v>
       </c>
@@ -6669,7 +6672,7 @@
         <v>21</v>
       </c>
       <c r="O98" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P98" s="13">
         <v>35884552807</v>
@@ -6681,7 +6684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>10379</v>
       </c>
@@ -6725,7 +6728,7 @@
         <v>21</v>
       </c>
       <c r="O99" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P99" s="13">
         <v>39183725881</v>
@@ -6737,7 +6740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>8932</v>
       </c>
@@ -6781,7 +6784,7 @@
         <v>21</v>
       </c>
       <c r="O100" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P100" s="13">
         <v>46067401835</v>
@@ -6793,7 +6796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:18" s="22" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:18" s="22" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="22">
         <v>8885</v>
       </c>
@@ -6837,7 +6840,7 @@
         <v>21</v>
       </c>
       <c r="O101" s="22" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P101" s="28">
         <v>15149756881</v>
@@ -6849,7 +6852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>10512</v>
       </c>
@@ -6893,7 +6896,7 @@
         <v>21</v>
       </c>
       <c r="O102" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P102" s="13">
         <v>35884552807</v>
@@ -6905,7 +6908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:18" s="22" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:18" s="22" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="22">
         <v>6338</v>
       </c>
@@ -6949,7 +6952,7 @@
         <v>21</v>
       </c>
       <c r="O103" s="22" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P103" s="28">
         <v>35538393844</v>
@@ -6961,7 +6964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>10451</v>
       </c>
@@ -7005,7 +7008,7 @@
         <v>21</v>
       </c>
       <c r="O104" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P104" s="13">
         <v>5673273533</v>
@@ -7017,7 +7020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>10537</v>
       </c>
@@ -7061,7 +7064,7 @@
         <v>21</v>
       </c>
       <c r="O105" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P105" s="13">
         <v>39183725881</v>
@@ -7073,7 +7076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>7689</v>
       </c>
@@ -7117,7 +7120,7 @@
         <v>21</v>
       </c>
       <c r="O106" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P106" s="13">
         <v>35538393844</v>
@@ -7129,7 +7132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>9293</v>
       </c>
@@ -7173,7 +7176,7 @@
         <v>21</v>
       </c>
       <c r="O107" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P107" s="13">
         <v>46067401835</v>
@@ -7185,7 +7188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>12915</v>
       </c>
@@ -7229,7 +7232,7 @@
         <v>21</v>
       </c>
       <c r="O108" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P108" s="13">
         <v>73368172549</v>
@@ -7241,7 +7244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:18" s="22" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:18" s="22" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="22">
         <v>10804</v>
       </c>
@@ -7285,7 +7288,7 @@
         <v>29</v>
       </c>
       <c r="O109" s="22" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P109" s="28">
         <v>73368172549</v>
@@ -7297,7 +7300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>6757</v>
       </c>
@@ -7341,7 +7344,7 @@
         <v>21</v>
       </c>
       <c r="O110" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P110" s="13">
         <v>35538393844</v>
@@ -7353,7 +7356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>13421</v>
       </c>
@@ -7397,7 +7400,7 @@
         <v>21</v>
       </c>
       <c r="O111" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P111" s="13">
         <v>46067401835</v>
@@ -7409,7 +7412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>6533</v>
       </c>
@@ -7453,7 +7456,7 @@
         <v>21</v>
       </c>
       <c r="O112" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P112" s="13">
         <v>46067401835</v>
@@ -7465,7 +7468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>6825</v>
       </c>
@@ -7509,7 +7512,7 @@
         <v>21</v>
       </c>
       <c r="O113" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P113" s="13">
         <v>73368172549</v>
@@ -7521,7 +7524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>346</v>
       </c>
@@ -7565,7 +7568,7 @@
         <v>21</v>
       </c>
       <c r="O114" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P114" s="13">
         <v>46067401835</v>
@@ -7577,7 +7580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>6300</v>
       </c>
@@ -7621,7 +7624,7 @@
         <v>21</v>
       </c>
       <c r="O115" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P115" s="13">
         <v>46067401835</v>
@@ -7633,7 +7636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>6021</v>
       </c>
@@ -7677,7 +7680,7 @@
         <v>21</v>
       </c>
       <c r="O116" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P116" s="13">
         <v>73368172549</v>
@@ -7689,7 +7692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:18" s="22" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:18" s="22" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="22">
         <v>5193</v>
       </c>
@@ -7733,7 +7736,7 @@
         <v>21</v>
       </c>
       <c r="O117" s="22" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P117" s="28">
         <v>46067401835</v>
@@ -7745,7 +7748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>8325</v>
       </c>
@@ -7789,7 +7792,7 @@
         <v>21</v>
       </c>
       <c r="O118" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P118" s="13">
         <v>35884552807</v>
@@ -7801,7 +7804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>5028</v>
       </c>
@@ -7845,7 +7848,7 @@
         <v>21</v>
       </c>
       <c r="O119" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P119" s="13">
         <v>73368172549</v>
@@ -7857,7 +7860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>7713</v>
       </c>
@@ -7901,7 +7904,7 @@
         <v>21</v>
       </c>
       <c r="O120" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P120" s="13">
         <v>39183725881</v>
@@ -7913,7 +7916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>11823</v>
       </c>
@@ -7957,7 +7960,7 @@
         <v>21</v>
       </c>
       <c r="O121" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P121" s="13">
         <v>35884552807</v>
@@ -7969,7 +7972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>5989</v>
       </c>
@@ -8013,7 +8016,7 @@
         <v>21</v>
       </c>
       <c r="O122" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P122" s="13">
         <v>46067401835</v>
@@ -8025,7 +8028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>10362</v>
       </c>
@@ -8069,7 +8072,7 @@
         <v>21</v>
       </c>
       <c r="O123" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P123" s="13">
         <v>33615887824</v>
@@ -8081,7 +8084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>13369</v>
       </c>
@@ -8125,7 +8128,7 @@
         <v>21</v>
       </c>
       <c r="O124" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P124" s="13">
         <v>33615887824</v>
@@ -8137,7 +8140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>6601</v>
       </c>
@@ -8181,7 +8184,7 @@
         <v>21</v>
       </c>
       <c r="O125" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P125" s="13">
         <v>73368172549</v>
@@ -8193,7 +8196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>13776</v>
       </c>
@@ -8231,7 +8234,7 @@
         <v>21</v>
       </c>
       <c r="O126" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P126" s="13">
         <v>73368172549</v>
@@ -8243,7 +8246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>8751</v>
       </c>
@@ -8287,7 +8290,7 @@
         <v>29</v>
       </c>
       <c r="O127" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P127" s="13">
         <v>73368172549</v>
@@ -8299,7 +8302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>8752</v>
       </c>
@@ -8343,7 +8346,7 @@
         <v>29</v>
       </c>
       <c r="O128" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P128" s="13">
         <v>73368172549</v>
@@ -8355,7 +8358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>8753</v>
       </c>
@@ -8399,7 +8402,7 @@
         <v>29</v>
       </c>
       <c r="O129" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P129" s="13">
         <v>73368172549</v>
@@ -8411,7 +8414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>13638</v>
       </c>
@@ -8449,7 +8452,7 @@
         <v>29</v>
       </c>
       <c r="O130" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P130" s="13">
         <v>33615887824</v>
@@ -8461,7 +8464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>10703</v>
       </c>
@@ -8505,7 +8508,7 @@
         <v>21</v>
       </c>
       <c r="O131" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P131" s="13">
         <v>73368172549</v>
@@ -8517,7 +8520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>8011</v>
       </c>
@@ -8561,7 +8564,7 @@
         <v>21</v>
       </c>
       <c r="O132" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P132" s="13">
         <v>35884552807</v>
@@ -8573,7 +8576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>13698</v>
       </c>
@@ -8617,7 +8620,7 @@
         <v>21</v>
       </c>
       <c r="O133" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P133" s="13">
         <v>39183725881</v>
@@ -8629,7 +8632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>13444</v>
       </c>
@@ -8673,7 +8676,7 @@
         <v>21</v>
       </c>
       <c r="O134" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P134" s="13">
         <v>15149756881</v>
@@ -8685,7 +8688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>7869</v>
       </c>
@@ -8729,7 +8732,7 @@
         <v>21</v>
       </c>
       <c r="O135" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P135" s="13">
         <v>35884552807</v>
@@ -8741,7 +8744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>8548</v>
       </c>
@@ -8785,7 +8788,7 @@
         <v>21</v>
       </c>
       <c r="O136" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P136" s="13">
         <v>39183725881</v>
@@ -8797,7 +8800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>11821</v>
       </c>
@@ -8841,7 +8844,7 @@
         <v>29</v>
       </c>
       <c r="O137" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P137" s="13">
         <v>35884552807</v>
@@ -8853,7 +8856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>13826</v>
       </c>
@@ -8897,7 +8900,7 @@
         <v>21</v>
       </c>
       <c r="O138" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P138" s="13">
         <v>33615887824</v>
@@ -8909,7 +8912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>12994</v>
       </c>
@@ -8953,7 +8956,7 @@
         <v>21</v>
       </c>
       <c r="O139" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P139" s="13">
         <v>35884552807</v>
@@ -8965,7 +8968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:18" s="22" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:18" s="22" customFormat="1" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="22">
         <v>8742</v>
       </c>
@@ -9009,7 +9012,7 @@
         <v>29</v>
       </c>
       <c r="O140" s="22" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P140" s="28">
         <v>35538393844</v>
@@ -9021,7 +9024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>13777</v>
       </c>
@@ -9059,7 +9062,7 @@
         <v>21</v>
       </c>
       <c r="O141" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P141" s="13">
         <v>39183725881</v>
@@ -9071,7 +9074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>13786</v>
       </c>
@@ -9109,7 +9112,7 @@
         <v>21</v>
       </c>
       <c r="O142" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P142" s="13">
         <v>39183725881</v>
@@ -9121,7 +9124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>13850</v>
       </c>
@@ -9165,7 +9168,7 @@
         <v>21</v>
       </c>
       <c r="O143" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P143" s="13" t="s">
         <v>38</v>
@@ -9174,7 +9177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>13302</v>
       </c>
@@ -9218,7 +9221,7 @@
         <v>21</v>
       </c>
       <c r="O144" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P144" s="13">
         <v>35884552807</v>
@@ -9230,7 +9233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>5866</v>
       </c>
@@ -9274,7 +9277,7 @@
         <v>21</v>
       </c>
       <c r="O145" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P145" s="13">
         <v>35884552807</v>
@@ -9286,7 +9289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>5442</v>
       </c>
@@ -9330,7 +9333,7 @@
         <v>21</v>
       </c>
       <c r="O146" t="s">
-        <v>24</v>
+        <v>228</v>
       </c>
       <c r="P146" s="13">
         <v>46067401835</v>
@@ -9342,7 +9345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>13221</v>
       </c>
@@ -9386,7 +9389,7 @@
         <v>21</v>
       </c>
       <c r="O147" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P147" s="13">
         <v>35884552807</v>
@@ -9398,7 +9401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>13857</v>
       </c>
@@ -9442,7 +9445,7 @@
         <v>21</v>
       </c>
       <c r="O148" t="s">
-        <v>22</v>
+        <v>228</v>
       </c>
       <c r="P148" s="13">
         <v>35884552807</v>
@@ -9454,7 +9457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>11151</v>
       </c>
@@ -9498,7 +9501,7 @@
         <v>21</v>
       </c>
       <c r="O149" t="s">
-        <v>61</v>
+        <v>228</v>
       </c>
       <c r="P149" s="13">
         <v>33615887824</v>
@@ -9510,7 +9513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>13864</v>
       </c>
@@ -9557,7 +9560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>13234</v>
       </c>
@@ -10363,7 +10366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>13813</v>
       </c>
@@ -11455,7 +11458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A186" s="14">
         <v>5341</v>
       </c>
@@ -12493,7 +12496,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:R204" xr:uid="{C64C195D-2B79-4C6D-852C-4F0C248DE140}">
-    <filterColumn colId="5">
+    <filterColumn colId="17">
       <filters>
         <filter val="VERDADEIRO"/>
       </filters>

</xml_diff>